<commit_message>
Verify the one-command claim and correct the timing
`make clean all` from an empty database: 4m28s, all 12 steps, 114 tests, 10 of
10 questions answered on the first attempt and matching the reference, DDR
rendered and verified at 2 pages. Every artefact in deliverables/ is from that
run.

The pipeline was estimated at "about six minutes" in the README, the DDR, the
workbook and the walkthrough notes. Measured, it is 4m28s, so all four now say
that instead - an estimate presented as a measurement is the same class of
mistake as an unverified number in a report.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165Za6gtPggDtMyRg2Z7ePj
</commit_message>
<xml_diff>
--- a/deliverables/Berka_TakeHome_Submission.xlsx
+++ b/deliverables/Berka_TakeHome_Submission.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-22T10:44:07+00:00</t>
+          <t>2026-10-22T10:55:22+00:00</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>95de493</t>
+          <t>b11c23f</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>make up &amp;&amp; make all (about 6 minutes end to end)</t>
+          <t>make up &amp;&amp; make all -- 4m28s end to end from an empty database</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>partner_bank and partner_account are both NULL; operation = NULL</t>
+          <t>partner_bank and partner_account are both NULL; operation = VKLAD</t>
         </is>
       </c>
     </row>
@@ -2593,19 +2593,19 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>SELECT region, count(*) AS client_count, round(100.0 * count(*) / sum(count(*)) OVER (), 2) AS pct_of_clients FROM ai.client GROUP BY region ORDER BY client_count DESC, region</t>
+          <t>SELECT region, count(*) AS client_count FROM ai.client GROUP BY region ORDER BY client_count DESC, region</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>region=south Moravia | client_count=937 | pct_of_clients=17.45
-region=north Moravia | client_count=920 | pct_of_clients=17.14
-region=central Bohemia | client_count=664 | pct_of_clients=12.37
-region=Prague | client_count=663 | pct_of_clients=12.35
-region=east Bohemia | client_count=660 | pct_of_clients=12.29
-region=north Bohemia | client_count=561 | pct_of_clients=10.45
-region=west Bohemia | client_count=515 | pct_of_clients=9.59
-region=south Bohemia | client_count=449 | pct_of_clients=8.36</t>
+          <t>region=south Moravia | client_count=937
+region=north Moravia | client_count=920
+region=central Bohemia | client_count=664
+region=Prague | client_count=663
+region=east Bohemia | client_count=660
+region=north Bohemia | client_count=561
+region=west Bohemia | client_count=515
+region=south Bohemia | client_count=449</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
@@ -2859,21 +2859,21 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>SELECT t.account_district_id, t.account_district_name, t.account_region, SUM(t.amount) AS incoming_amount_czk, COUNT(*) AS credit_posting_count, COUNT(DISTINCT t.account_id) AS accounts_with_credits FROM ai.transaction t WHERE t.direction = 'credit' AND t.trans_date &gt;= DATE '1997-01-01' AND t.trans_date &lt; DATE '1998-01-01' GROUP BY t.account_district_id, t.account_district_name, t.account_region ORDER BY incoming_amount_czk DESC, t.account_district_name ASC LIMIT 10</t>
+          <t>SELECT account_district_id AS district_id, account_district_name AS district_name, account_region AS region, sum(amount) AS total_incoming_amount, count(*) AS credit_posting_count, count(DISTINCT account_id) AS account_count FROM ai.transaction WHERE direction = 'credit' AND trans_date &gt;= DATE '1997-01-01' AND trans_date &lt; DATE '1998-01-01' GROUP BY account_district_id, account_district_name, account_region ORDER BY sum(amount) DESC, account_district_id LIMIT 10</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>account_district_id=1 | account_district_name=Hl.m. Praha | account_region=Prague | incoming_amount_czk=115130200.1 | credit_posting_count=13611 | accounts_with_credits=554
-account_district_id=70 | account_district_name=Karvina | account_region=north Moravia | incoming_amount_czk=28506437.1 | credit_posting_count=3802 | accounts_with_credits=152
-account_district_id=74 | account_district_name=Ostrava - mesto | account_region=north Moravia | incoming_amount_czk=27689271.9 | credit_posting_count=3378 | accounts_with_credits=135
-account_district_id=54 | account_district_name=Brno - mesto | account_region=south Moravia | incoming_amount_czk=23095083.4 | credit_posting_count=3041 | accounts_with_credits=128
-account_district_id=64 | account_district_name=Zlin | account_region=south Moravia | incoming_amount_czk=19723168.5 | credit_posting_count=2299 | accounts_with_credits=92
-account_district_id=68 | account_district_name=Frydek - Mistek | account_region=north Moravia | incoming_amount_czk=19087598.8 | credit_posting_count=2006 | accounts_with_credits=83
-account_district_id=72 | account_district_name=Olomouc | account_region=north Moravia | incoming_amount_czk=15916397.0 | credit_posting_count=2129 | accounts_with_credits=88
-account_district_id=5 | account_district_name=Kolin | account_region=central Bohemia | incoming_amount_czk=14471603.6 | credit_posting_count=1542 | accounts_with_credits=65
-account_district_id=52 | account_district_name=Usti nad Orlici | account_region=east Bohemia | incoming_amount_czk=14085167.4 | credit_posting_count=1431 | accounts_with_credits=57
-account_district_id=19 | account_district_name=Prachatice | account_region=south Bohemia | incoming_amount_czk=12163147.0 | credit_posting_count=1359 | accounts_with_credits=55</t>
+          <t>district_id=1 | district_name=Hl.m. Praha | region=Prague | total_incoming_amount=115130200.1 | credit_posting_count=13611 | account_count=554
+district_id=70 | district_name=Karvina | region=north Moravia | total_incoming_amount=28506437.1 | credit_posting_count=3802 | account_count=152
+district_id=74 | district_name=Ostrava - mesto | region=north Moravia | total_incoming_amount=27689271.9 | credit_posting_count=3378 | account_count=135
+district_id=54 | district_name=Brno - mesto | region=south Moravia | total_incoming_amount=23095083.4 | credit_posting_count=3041 | account_count=128
+district_id=64 | district_name=Zlin | region=south Moravia | total_incoming_amount=19723168.5 | credit_posting_count=2299 | account_count=92
+district_id=68 | district_name=Frydek - Mistek | region=north Moravia | total_incoming_amount=19087598.8 | credit_posting_count=2006 | account_count=83
+district_id=72 | district_name=Olomouc | region=north Moravia | total_incoming_amount=15916397.0 | credit_posting_count=2129 | account_count=88
+district_id=5 | district_name=Kolin | region=central Bohemia | total_incoming_amount=14471603.6 | credit_posting_count=1542 | account_count=65
+district_id=52 | district_name=Usti nad Orlici | region=east Bohemia | total_incoming_amount=14085167.4 | credit_posting_count=1431 | account_count=57
+district_id=19 | district_name=Prachatice | region=south Bohemia | total_incoming_amount=12163147.0 | credit_posting_count=1359 | account_count=55</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>SELECT c.year_month AS month, c.month_start AS month_start, COUNT(a.account_id) AS new_accounts FROM ai.calendar c LEFT JOIN ai.account a ON a.open_date = c.date_key WHERE c.year = 1996 GROUP BY c.year_month, c.month_start ORDER BY c.month_start</t>
+          <t>SELECT c.year_month AS month, c.month_start AS month_start, count(a.account_id) AS new_accounts FROM ai.calendar c LEFT JOIN ai.account a ON a.open_date = c.date_key WHERE c.year = 1996 GROUP BY c.year_month, c.month_start ORDER BY c.month_start</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -3015,15 +3015,15 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>SELECT loan_status, status_code, count(*) AS loan_count, round(avg(owner_age_at_loan_start), 2) AS average_age_at_loan_start, count(*) FILTER (WHERE data_quality_flags @&gt; ARRAY['val_owner_age_at_loan_start']) AS under_15_flagged_loans, round(avg(owner_age_at_loan_start) FILTER (WHERE NOT (data_quality_flags @&gt; ARRAY['val_owner_age_at_loan_start'])), 2) AS average_age_excluding_flagged FROM ai.loan GROUP BY loan_status, status_code ORDER BY status_code</t>
+          <t>SELECT loan_status, count(*) AS loan_count, round(avg(owner_age_at_loan_start), 2) AS average_age_at_loan_start, count(*) FILTER (WHERE 'val_owner_age_at_loan_start' = ANY(data_quality_flags)) AS flagged_under_15_loans, round(avg(owner_age_at_loan_start) FILTER (WHERE NOT ('val_owner_age_at_loan_start' = ANY(data_quality_flags))), 2) AS average_age_excluding_flagged FROM ai.loan GROUP BY loan_status ORDER BY loan_status</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>loan_status=finished, paid in full | status_code=A | loan_count=203 | average_age_at_loan_start=37.07 | under_15_flagged_loans=4 | average_age_excluding_flagged=37.53
-loan_status=finished, unpaid (default) | status_code=B | loan_count=31 | average_age_at_loan_start=39.61 | under_15_flagged_loans=0 | average_age_excluding_flagged=39.61
-loan_status=running, no problem | status_code=C | loan_count=403 | average_age_at_loan_start=38.7 | under_15_flagged_loans=2 | average_age_excluding_flagged=38.82
-loan_status=running, client in debt | status_code=D | loan_count=45 | average_age_at_loan_start=37.0 | under_15_flagged_loans=0 | average_age_excluding_flagged=37.0</t>
+          <t>loan_status=finished, paid in full | loan_count=203 | average_age_at_loan_start=37.07 | flagged_under_15_loans=4 | average_age_excluding_flagged=37.53
+loan_status=finished, unpaid (default) | loan_count=31 | average_age_at_loan_start=39.61 | flagged_under_15_loans=0 | average_age_excluding_flagged=39.61
+loan_status=running, client in debt | loan_count=45 | average_age_at_loan_start=37.0 | flagged_under_15_loans=0 | average_age_excluding_flagged=37.0
+loan_status=running, no problem | loan_count=403 | average_age_at_loan_start=38.7 | flagged_under_15_loans=2 | average_age_excluding_flagged=38.82</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
@@ -3076,13 +3076,13 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>SELECT owner_gender AS gender, count(*) AS owner_count, sum(count(*)) OVER () AS total_gold_owners, round(100.0 * count(*) / sum(count(*)) OVER (), 2) AS share_pct FROM ai.account_owner WHERE owner_card_type = 'gold' GROUP BY owner_gender ORDER BY owner_gender</t>
+          <t>SELECT owner_gender AS gender, count(*) AS owner_count, round(100.0 * count(*) / sum(count(*)) OVER (), 2) AS share_pct, sum(count(*)) OVER () AS total_gold_card_owners FROM ai.account_owner WHERE owner_card_type = 'gold' GROUP BY owner_gender ORDER BY owner_gender</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>gender=female | owner_count=35 | total_gold_owners=88.0 | share_pct=39.77
-gender=male | owner_count=53 | total_gold_owners=88.0 | share_pct=60.23</t>
+          <t>gender=female | owner_count=35 | share_pct=39.77 | total_gold_card_owners=88.0
+gender=male | owner_count=53 | share_pct=60.23 | total_gold_card_owners=88.0</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
@@ -3138,12 +3138,12 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>SELECT round(avg(closing_balance), 2) AS average_month_end_balance, count(*) AS accounts_with_balance, count(*) FILTER (WHERE is_carried_forward) AS carried_forward_balances, count(*) FILTER (WHERE 'con_balance_reconciliation_material' = ANY(account_data_quality_flags)) AS accounts_with_reconciliation_flag FROM ai.account_month_end_balance WHERE month_end_date = DATE '1998-12-31'</t>
+          <t>SELECT round(avg(closing_balance), 2) AS average_month_end_balance, count(*) AS accounts_with_balance, count(*) FILTER (WHERE is_carried_forward) AS carried_forward_balances FROM ai.account_month_end_balance WHERE month_end_date = DATE '1998-12-31'</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>average_month_end_balance=43808.94 | accounts_with_balance=4500 | carried_forward_balances=76 | accounts_with_reconciliation_flag=55</t>
+          <t>average_month_end_balance=43808.94 | accounts_with_balance=4500 | carried_forward_balances=76</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
@@ -3413,11 +3413,6 @@
           <t>client_count</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>pct_of_clients</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
@@ -3428,9 +3423,6 @@
       <c r="B17" s="15" t="n">
         <v>937</v>
       </c>
-      <c r="C17" s="15" t="n">
-        <v>17.45</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
@@ -3441,9 +3433,6 @@
       <c r="B18" s="15" t="n">
         <v>920</v>
       </c>
-      <c r="C18" s="15" t="n">
-        <v>17.14</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
@@ -3454,9 +3443,6 @@
       <c r="B19" s="15" t="n">
         <v>664</v>
       </c>
-      <c r="C19" s="15" t="n">
-        <v>12.37</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
@@ -3467,9 +3453,6 @@
       <c r="B20" s="15" t="n">
         <v>663</v>
       </c>
-      <c r="C20" s="15" t="n">
-        <v>12.35</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
@@ -3480,9 +3463,6 @@
       <c r="B21" s="15" t="n">
         <v>660</v>
       </c>
-      <c r="C21" s="15" t="n">
-        <v>12.29</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
@@ -3493,9 +3473,6 @@
       <c r="B22" s="15" t="n">
         <v>561</v>
       </c>
-      <c r="C22" s="15" t="n">
-        <v>10.45</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
@@ -3506,9 +3483,6 @@
       <c r="B23" s="15" t="n">
         <v>515</v>
       </c>
-      <c r="C23" s="15" t="n">
-        <v>9.59</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
@@ -3518,9 +3492,6 @@
       </c>
       <c r="B24" s="15" t="n">
         <v>449</v>
-      </c>
-      <c r="C24" s="15" t="n">
-        <v>8.359999999999999</v>
       </c>
     </row>
     <row r="27">
@@ -4333,22 +4304,22 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>account_district_id</t>
+          <t>district_id</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>account_district_name</t>
+          <t>district_name</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>account_region</t>
+          <t>region</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>incoming_amount_czk</t>
+          <t>total_incoming_amount</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -4358,7 +4329,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>accounts_with_credits</t>
+          <t>account_count</t>
         </is>
       </c>
     </row>
@@ -5232,25 +5203,20 @@
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>status_code</t>
+          <t>loan_count</t>
         </is>
       </c>
       <c r="C142" s="5" t="inlineStr">
         <is>
-          <t>loan_count</t>
+          <t>average_age_at_loan_start</t>
         </is>
       </c>
       <c r="D142" s="5" t="inlineStr">
         <is>
-          <t>average_age_at_loan_start</t>
+          <t>flagged_under_15_loans</t>
         </is>
       </c>
       <c r="E142" s="5" t="inlineStr">
-        <is>
-          <t>under_15_flagged_loans</t>
-        </is>
-      </c>
-      <c r="F142" s="5" t="inlineStr">
         <is>
           <t>average_age_excluding_flagged</t>
         </is>
@@ -5262,21 +5228,16 @@
           <t>finished, paid in full</t>
         </is>
       </c>
-      <c r="B143" s="15" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
+      <c r="B143" s="15" t="n">
+        <v>203</v>
       </c>
       <c r="C143" s="15" t="n">
-        <v>203</v>
+        <v>37.07</v>
       </c>
       <c r="D143" s="15" t="n">
-        <v>37.07</v>
+        <v>4</v>
       </c>
       <c r="E143" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="F143" s="15" t="n">
         <v>37.53</v>
       </c>
     </row>
@@ -5286,70 +5247,55 @@
           <t>finished, unpaid (default)</t>
         </is>
       </c>
-      <c r="B144" s="15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+      <c r="B144" s="15" t="n">
+        <v>31</v>
       </c>
       <c r="C144" s="15" t="n">
-        <v>31</v>
+        <v>39.61</v>
       </c>
       <c r="D144" s="15" t="n">
-        <v>39.61</v>
+        <v>0</v>
       </c>
       <c r="E144" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F144" s="15" t="n">
         <v>39.61</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="15" t="inlineStr">
         <is>
-          <t>running, no problem</t>
-        </is>
-      </c>
-      <c r="B145" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+          <t>running, client in debt</t>
+        </is>
+      </c>
+      <c r="B145" s="15" t="n">
+        <v>45</v>
       </c>
       <c r="C145" s="15" t="n">
-        <v>403</v>
+        <v>37</v>
       </c>
       <c r="D145" s="15" t="n">
-        <v>38.7</v>
+        <v>0</v>
       </c>
       <c r="E145" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F145" s="15" t="n">
-        <v>38.82</v>
+        <v>37</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="15" t="inlineStr">
         <is>
-          <t>running, client in debt</t>
-        </is>
-      </c>
-      <c r="B146" s="15" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
+          <t>running, no problem</t>
+        </is>
+      </c>
+      <c r="B146" s="15" t="n">
+        <v>403</v>
       </c>
       <c r="C146" s="15" t="n">
-        <v>45</v>
+        <v>38.7</v>
       </c>
       <c r="D146" s="15" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E146" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F146" s="15" t="n">
-        <v>37</v>
+        <v>38.82</v>
       </c>
     </row>
     <row r="149">
@@ -5440,12 +5386,12 @@
       </c>
       <c r="C156" s="5" t="inlineStr">
         <is>
-          <t>total_gold_owners</t>
+          <t>share_pct</t>
         </is>
       </c>
       <c r="D156" s="5" t="inlineStr">
         <is>
-          <t>share_pct</t>
+          <t>total_gold_card_owners</t>
         </is>
       </c>
     </row>
@@ -5459,10 +5405,10 @@
         <v>35</v>
       </c>
       <c r="C157" s="15" t="n">
+        <v>39.77</v>
+      </c>
+      <c r="D157" s="15" t="n">
         <v>88</v>
-      </c>
-      <c r="D157" s="15" t="n">
-        <v>39.77</v>
       </c>
     </row>
     <row r="158">
@@ -5475,10 +5421,10 @@
         <v>53</v>
       </c>
       <c r="C158" s="15" t="n">
+        <v>60.23</v>
+      </c>
+      <c r="D158" s="15" t="n">
         <v>88</v>
-      </c>
-      <c r="D158" s="15" t="n">
-        <v>60.23</v>
       </c>
     </row>
     <row r="161">
@@ -5586,11 +5532,6 @@
           <t>carried_forward_balances</t>
         </is>
       </c>
-      <c r="D167" s="5" t="inlineStr">
-        <is>
-          <t>accounts_with_reconciliation_flag</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" s="15" t="n">
@@ -5601,9 +5542,6 @@
       </c>
       <c r="C168" s="15" t="n">
         <v>76</v>
-      </c>
-      <c r="D168" s="15" t="n">
-        <v>55</v>
       </c>
     </row>
     <row r="171">
@@ -10916,7 +10854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -11438,6 +11376,402 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>workbook</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>make workbook</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:44:08+00:00</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>{"tabs": ["Overview", "Defect types", "Model", "Questions", "Q detail", "DQ rules", "Assumptions", "Entitlements", "Run log"], "defect_types": 14}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>make zip</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:45:18+00:00</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>{"files": 74, "size_kb": 469.7}</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>ddr</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>make ddr</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:47:20+00:00</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>{"words": 1520, "pages": 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>make zip</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:49:22+00:00</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>{"files": 79, "size_kb": 483.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>ingest</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>make ingest</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:50:34+00:00</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>{"run_id": "bd7b7fd2-e741-459c-90ed-f1ce8a1b4fc8", "row_counts": {"account": 4500, "client": 5369, "disp": 5369, "card": 892, "loan": 682, "order": 6471, "trans": 1056320, "district": 77}, "mismatches": []}</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>make profile</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:51:36+00:00</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>{"tables": {"district": 77, "client": 5369, "account": 4500, "disp": 5369, "card": 892, "loan": 682, "order": 6471, "trans": 1056320}, "candidates_present": 13, "candidates_total": 17}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>dq</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>make dq (dataset=stg)</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:51:53+00:00</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>{"run_id": "55ac5752-e529-4ad3-b3b6-2723e5a50227", "dataset": "stg", "rules_executed": 123, "rules_fired": 19, "rules_errored": 0, "by_severity": {"block": 1, "warn": 6, "info": 12}, "rows_quarantined": 1, "quarantined_by_table": {"trans": 1}, "rows_flagged": 440, "flagged_by_table": {"account": 0, "client": 114, "disp": 0, "card": 0, "loan": 6, "trans": 320, "district": 0, "order": 0, "all": 0}, "duration_sec": 16.24, "defect_types": 14}</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>make model</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:52:04+00:00</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>{"row_counts": {"dim_date": 2191, "dim_district": 77, "dim_client": 5369, "dim_account": 4500, "bridge_disposition": 5369, "dim_card": 892, "fact_loan": 682, "fact_transaction": 1056319, "fact_account_month_end_balance": 185615}, "ref_codes": 27, "problems": [], "reconciliation_checks": 9}</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>entitlements</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>make entitlements</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:52:05+00:00</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>{"policies": 7, "visible_rows": [{"db_role": "cro_global", "display_name": "Group risk, bank-wide reporting", "clients": 5369, "accounts": 4500, "loans": 682, "transactions": 1056319, "districts": 77, "portfolios": "ALL_CLIENTS"}, {"db_role": "rm_north", "display_name": "Relationship manager, northern book", "clients": 1481, "accounts": 1241, "loans": 179, "transactions": 294622, "districts": 77, "portfolios": "NORTH_BOOK"}, {"db_role": "rm_south", "display_name": "Relationship manager, southern book", "clients": 1386, "accounts": 1157, "loans": 194, "transactions": 272331, "districts": 77, "portfolios": "SOUTH_BOOK"}, {"db_role": "rm_unassigned", "display_name": "Newly created user with no portfolio yet", "clients": 0, "accounts": 0, "loans": 0, "transactions": 0, "districts": 77, "portfolios": null}]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>make reference</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:52:05+00:00</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>{"questions": 10, "failures": []}</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>semantic</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>make semantic</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:52:07+00:00</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>{"entities": 11, "columns": 100, "context_pack_chars": 27592, "problems": []}</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>entitlements</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>make entitlements</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:52:08+00:00</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>{"policies": 7, "visible_rows": [{"db_role": "cro_global", "display_name": "Group risk, bank-wide reporting", "clients": 5369, "accounts": 4500, "loans": 682, "transactions": 1056319, "districts": 77, "portfolios": "ALL_CLIENTS"}, {"db_role": "rm_north", "display_name": "Relationship manager, northern book", "clients": 1481, "accounts": 1241, "loans": 179, "transactions": 294622, "districts": 77, "portfolios": "NORTH_BOOK"}, {"db_role": "rm_south", "display_name": "Relationship manager, southern book", "clients": 1386, "accounts": 1157, "loans": 194, "transactions": 272331, "districts": 77, "portfolios": "SOUTH_BOOK"}, {"db_role": "rm_unassigned", "display_name": "Newly created user with no portfolio yet", "clients": 0, "accounts": 0, "loans": 0, "transactions": 0, "districts": 77, "portfolios": null}]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>questions</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>make questions (provider=claude_cli, model=claude-sonnet-5-5)</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:54:03+00:00</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>{"answered": 10, "total": 10, "answered_first_attempt": 10, "run_as": "cro_global"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>evaluate</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>make evaluate</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:54:04+00:00</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>{"tally": {"match": 10}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>workbook</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>make workbook</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:54:55+00:00</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>{"tabs": ["Overview", "Defect types", "Model", "Questions", "Q detail", "DQ rules", "Assumptions", "Entitlements", "Run log"], "defect_types": 14}</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>ddr</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>make ddr</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:54:57+00:00</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>{"words": 1520, "pages": 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>make zip</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:54:57+00:00</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>{"files": 79, "size_kb": 482.3}</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>ddr</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>make ddr</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22T10:55:21+00:00</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>{"words": 1527, "pages": 2}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>